<commit_message>
refactor: Rewrite DBC clone to INSERT SET format, sync item DBC (F-044)
- Clone now emits INSERT SET with only non-default values
- Clean float precision in cloned spells
- Item DBC sync: 8 new items added (489 total)
- Remove obsolete Extra Icons scripts
- Update Race and Class Masks spreadsheet

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cli/data/Race and Class Masks.xlsx
+++ b/cli/data/Race and Class Masks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\wow-server\Zeppelin-Craft\Scripts\Starting Weapons\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\wow-server\Zeppelin-Craft\cli\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA0AD78-6557-4325-8B5A-3E90C2C17373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6540A246-8E3B-4A28-88B9-2D31C69CD43F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1716" yWindow="3960" windowWidth="21624" windowHeight="18456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10320" yWindow="5628" windowWidth="34560" windowHeight="18648" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Race Mask" sheetId="1" r:id="rId1"/>
@@ -22,17 +22,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Weapon Class Mask'!$A$3:$B$3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -756,16 +745,16 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -790,146 +779,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1027,6 +876,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
@@ -1041,7 +897,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1049,6 +905,20 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1070,6 +940,125 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1697,11 +1686,11 @@
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="15"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="1">
         <f>SUM(E2:E13)</f>
         <v>3039</v>
@@ -1890,11 +1879,11 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="15"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="1">
         <f>SUM(D2:D11)</f>
         <v>1023</v>
@@ -1920,10 +1909,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="15"/>
+      <c r="A1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="18"/>
       <c r="C1" s="1">
         <v>1</v>
       </c>
@@ -1959,10 +1948,10 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="18"/>
       <c r="C2" s="1">
         <f t="shared" ref="C2:L2" si="0">POWER(2,C1-1)</f>
         <v>1</v>
@@ -2377,12 +2366,12 @@
       <c r="K11" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="L11" s="5" t="b">
-        <v>0</v>
+      <c r="L11" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="M11" s="3">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -2777,28 +2766,28 @@
     <cfRule type="cellIs" dxfId="43" priority="268" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="267">
+    <cfRule type="cellIs" dxfId="42" priority="265" operator="equal">
+      <formula>"LEARN"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="267">
       <formula>AND(C4=FALSE, C4&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="266">
+    <cfRule type="expression" dxfId="40" priority="266">
       <formula>"INVALID"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="265" operator="equal">
-      <formula>"LEARN"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:G18">
     <cfRule type="cellIs" dxfId="39" priority="212" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="209" operator="equal">
-      <formula>"LEARN"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="37" priority="211">
+    <cfRule type="expression" dxfId="38" priority="211">
       <formula>AND(F4=FALSE, F4&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="210">
+    <cfRule type="expression" dxfId="37" priority="210">
       <formula>"INVALID"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="209" operator="equal">
+      <formula>"LEARN"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F19:L20">
@@ -2833,28 +2822,28 @@
     <cfRule type="cellIs" dxfId="27" priority="41" operator="equal">
       <formula>"LEARN"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="42">
-      <formula>"INVALID"</formula>
+    <cfRule type="cellIs" dxfId="26" priority="44" operator="equal">
+      <formula>TRUE</formula>
     </cfRule>
     <cfRule type="expression" dxfId="25" priority="43">
       <formula>AND(H4=FALSE, H4&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="44" operator="equal">
-      <formula>TRUE</formula>
+    <cfRule type="expression" dxfId="24" priority="42">
+      <formula>"INVALID"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I8:I18">
     <cfRule type="cellIs" dxfId="23" priority="149" operator="equal">
       <formula>"LEARN"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="152" operator="equal">
-      <formula>TRUE</formula>
+    <cfRule type="expression" dxfId="22" priority="150">
+      <formula>"INVALID"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="21" priority="151">
       <formula>AND(I8=FALSE, I8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="150">
-      <formula>"INVALID"</formula>
+    <cfRule type="cellIs" dxfId="20" priority="152" operator="equal">
+      <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:K7">
@@ -2872,17 +2861,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J8:K12">
-    <cfRule type="cellIs" dxfId="15" priority="57" operator="equal">
-      <formula>"LEARN"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="58">
+    <cfRule type="expression" dxfId="15" priority="58">
       <formula>"INVALID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="59">
+    <cfRule type="expression" dxfId="14" priority="59">
       <formula>AND(J8=FALSE, J8&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="60" operator="equal">
       <formula>TRUE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="57" operator="equal">
+      <formula>"LEARN"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J13:L18">
@@ -2900,17 +2889,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L12">
-    <cfRule type="expression" dxfId="7" priority="22">
+    <cfRule type="cellIs" dxfId="7" priority="21" operator="equal">
+      <formula>"LEARN"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="22">
       <formula>"INVALID"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="23">
+    <cfRule type="expression" dxfId="5" priority="23">
       <formula>AND(L5=FALSE, L5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
       <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="21" operator="equal">
-      <formula>"LEARN"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2938,19 +2927,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="18"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -3543,19 +3532,19 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="18"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="15"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -4093,19 +4082,19 @@
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="18"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="15"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
@@ -4643,19 +4632,19 @@
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A51" s="16" t="s">
+      <c r="A51" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="17"/>
-      <c r="C51" s="17"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="17"/>
-      <c r="I51" s="17"/>
-      <c r="J51" s="17"/>
-      <c r="K51" s="18"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="14"/>
+      <c r="K51" s="15"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
@@ -5193,19 +5182,19 @@
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="16" t="s">
+      <c r="A68" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B68" s="17"/>
-      <c r="C68" s="17"/>
-      <c r="D68" s="17"/>
-      <c r="E68" s="17"/>
-      <c r="F68" s="17"/>
-      <c r="G68" s="17"/>
-      <c r="H68" s="17"/>
-      <c r="I68" s="17"/>
-      <c r="J68" s="17"/>
-      <c r="K68" s="18"/>
+      <c r="B68" s="14"/>
+      <c r="C68" s="14"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="14"/>
+      <c r="F68" s="14"/>
+      <c r="G68" s="14"/>
+      <c r="H68" s="14"/>
+      <c r="I68" s="14"/>
+      <c r="J68" s="14"/>
+      <c r="K68" s="15"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" s="10" t="s">
@@ -5743,19 +5732,19 @@
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A85" s="16" t="s">
+      <c r="A85" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B85" s="17"/>
-      <c r="C85" s="17"/>
-      <c r="D85" s="17"/>
-      <c r="E85" s="17"/>
-      <c r="F85" s="17"/>
-      <c r="G85" s="17"/>
-      <c r="H85" s="17"/>
-      <c r="I85" s="17"/>
-      <c r="J85" s="17"/>
-      <c r="K85" s="18"/>
+      <c r="B85" s="14"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="14"/>
+      <c r="G85" s="14"/>
+      <c r="H85" s="14"/>
+      <c r="I85" s="14"/>
+      <c r="J85" s="14"/>
+      <c r="K85" s="15"/>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86" s="10" t="s">
@@ -6293,19 +6282,19 @@
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A102" s="16" t="s">
+      <c r="A102" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B102" s="17"/>
-      <c r="C102" s="17"/>
-      <c r="D102" s="17"/>
-      <c r="E102" s="17"/>
-      <c r="F102" s="17"/>
-      <c r="G102" s="17"/>
-      <c r="H102" s="17"/>
-      <c r="I102" s="17"/>
-      <c r="J102" s="17"/>
-      <c r="K102" s="18"/>
+      <c r="B102" s="14"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="14"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="14"/>
+      <c r="G102" s="14"/>
+      <c r="H102" s="14"/>
+      <c r="I102" s="14"/>
+      <c r="J102" s="14"/>
+      <c r="K102" s="15"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" s="10" t="s">
@@ -6843,19 +6832,19 @@
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A119" s="16" t="s">
+      <c r="A119" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="B119" s="17"/>
-      <c r="C119" s="17"/>
-      <c r="D119" s="17"/>
-      <c r="E119" s="17"/>
-      <c r="F119" s="17"/>
-      <c r="G119" s="17"/>
-      <c r="H119" s="17"/>
-      <c r="I119" s="17"/>
-      <c r="J119" s="17"/>
-      <c r="K119" s="18"/>
+      <c r="B119" s="14"/>
+      <c r="C119" s="14"/>
+      <c r="D119" s="14"/>
+      <c r="E119" s="14"/>
+      <c r="F119" s="14"/>
+      <c r="G119" s="14"/>
+      <c r="H119" s="14"/>
+      <c r="I119" s="14"/>
+      <c r="J119" s="14"/>
+      <c r="K119" s="15"/>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120" s="10" t="s">
@@ -7393,19 +7382,19 @@
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A136" s="16" t="s">
+      <c r="A136" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B136" s="17"/>
-      <c r="C136" s="17"/>
-      <c r="D136" s="17"/>
-      <c r="E136" s="17"/>
-      <c r="F136" s="17"/>
-      <c r="G136" s="17"/>
-      <c r="H136" s="17"/>
-      <c r="I136" s="17"/>
-      <c r="J136" s="17"/>
-      <c r="K136" s="18"/>
+      <c r="B136" s="14"/>
+      <c r="C136" s="14"/>
+      <c r="D136" s="14"/>
+      <c r="E136" s="14"/>
+      <c r="F136" s="14"/>
+      <c r="G136" s="14"/>
+      <c r="H136" s="14"/>
+      <c r="I136" s="14"/>
+      <c r="J136" s="14"/>
+      <c r="K136" s="15"/>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="10" t="s">
@@ -7943,19 +7932,19 @@
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A153" s="16" t="s">
+      <c r="A153" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B153" s="17"/>
-      <c r="C153" s="17"/>
-      <c r="D153" s="17"/>
-      <c r="E153" s="17"/>
-      <c r="F153" s="17"/>
-      <c r="G153" s="17"/>
-      <c r="H153" s="17"/>
-      <c r="I153" s="17"/>
-      <c r="J153" s="17"/>
-      <c r="K153" s="18"/>
+      <c r="B153" s="14"/>
+      <c r="C153" s="14"/>
+      <c r="D153" s="14"/>
+      <c r="E153" s="14"/>
+      <c r="F153" s="14"/>
+      <c r="G153" s="14"/>
+      <c r="H153" s="14"/>
+      <c r="I153" s="14"/>
+      <c r="J153" s="14"/>
+      <c r="K153" s="15"/>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154" s="10" t="s">
@@ -8493,19 +8482,19 @@
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A170" s="16" t="s">
+      <c r="A170" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B170" s="17"/>
-      <c r="C170" s="17"/>
-      <c r="D170" s="17"/>
-      <c r="E170" s="17"/>
-      <c r="F170" s="17"/>
-      <c r="G170" s="17"/>
-      <c r="H170" s="17"/>
-      <c r="I170" s="17"/>
-      <c r="J170" s="17"/>
-      <c r="K170" s="18"/>
+      <c r="B170" s="14"/>
+      <c r="C170" s="14"/>
+      <c r="D170" s="14"/>
+      <c r="E170" s="14"/>
+      <c r="F170" s="14"/>
+      <c r="G170" s="14"/>
+      <c r="H170" s="14"/>
+      <c r="I170" s="14"/>
+      <c r="J170" s="14"/>
+      <c r="K170" s="15"/>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A171" s="10" t="s">
@@ -9043,19 +9032,19 @@
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A187" s="16" t="s">
+      <c r="A187" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B187" s="17"/>
-      <c r="C187" s="17"/>
-      <c r="D187" s="17"/>
-      <c r="E187" s="17"/>
-      <c r="F187" s="17"/>
-      <c r="G187" s="17"/>
-      <c r="H187" s="17"/>
-      <c r="I187" s="17"/>
-      <c r="J187" s="17"/>
-      <c r="K187" s="18"/>
+      <c r="B187" s="14"/>
+      <c r="C187" s="14"/>
+      <c r="D187" s="14"/>
+      <c r="E187" s="14"/>
+      <c r="F187" s="14"/>
+      <c r="G187" s="14"/>
+      <c r="H187" s="14"/>
+      <c r="I187" s="14"/>
+      <c r="J187" s="14"/>
+      <c r="K187" s="15"/>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A188" s="10" t="s">
@@ -9593,19 +9582,19 @@
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A204" s="16" t="s">
+      <c r="A204" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B204" s="17"/>
-      <c r="C204" s="17"/>
-      <c r="D204" s="17"/>
-      <c r="E204" s="17"/>
-      <c r="F204" s="17"/>
-      <c r="G204" s="17"/>
-      <c r="H204" s="17"/>
-      <c r="I204" s="17"/>
-      <c r="J204" s="17"/>
-      <c r="K204" s="18"/>
+      <c r="B204" s="14"/>
+      <c r="C204" s="14"/>
+      <c r="D204" s="14"/>
+      <c r="E204" s="14"/>
+      <c r="F204" s="14"/>
+      <c r="G204" s="14"/>
+      <c r="H204" s="14"/>
+      <c r="I204" s="14"/>
+      <c r="J204" s="14"/>
+      <c r="K204" s="15"/>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A205" s="10" t="s">
@@ -10143,19 +10132,19 @@
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A221" s="16" t="s">
+      <c r="A221" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="B221" s="17"/>
-      <c r="C221" s="17"/>
-      <c r="D221" s="17"/>
-      <c r="E221" s="17"/>
-      <c r="F221" s="17"/>
-      <c r="G221" s="17"/>
-      <c r="H221" s="17"/>
-      <c r="I221" s="17"/>
-      <c r="J221" s="17"/>
-      <c r="K221" s="18"/>
+      <c r="B221" s="14"/>
+      <c r="C221" s="14"/>
+      <c r="D221" s="14"/>
+      <c r="E221" s="14"/>
+      <c r="F221" s="14"/>
+      <c r="G221" s="14"/>
+      <c r="H221" s="14"/>
+      <c r="I221" s="14"/>
+      <c r="J221" s="14"/>
+      <c r="K221" s="15"/>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A222" s="10" t="s">
@@ -10693,19 +10682,19 @@
       </c>
     </row>
     <row r="238" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A238" s="16" t="s">
+      <c r="A238" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B238" s="17"/>
-      <c r="C238" s="17"/>
-      <c r="D238" s="17"/>
-      <c r="E238" s="17"/>
-      <c r="F238" s="17"/>
-      <c r="G238" s="17"/>
-      <c r="H238" s="17"/>
-      <c r="I238" s="17"/>
-      <c r="J238" s="17"/>
-      <c r="K238" s="18"/>
+      <c r="B238" s="14"/>
+      <c r="C238" s="14"/>
+      <c r="D238" s="14"/>
+      <c r="E238" s="14"/>
+      <c r="F238" s="14"/>
+      <c r="G238" s="14"/>
+      <c r="H238" s="14"/>
+      <c r="I238" s="14"/>
+      <c r="J238" s="14"/>
+      <c r="K238" s="15"/>
     </row>
     <row r="239" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A239" s="10" t="s">
@@ -11243,19 +11232,19 @@
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A255" s="16" t="s">
+      <c r="A255" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B255" s="17"/>
-      <c r="C255" s="17"/>
-      <c r="D255" s="17"/>
-      <c r="E255" s="17"/>
-      <c r="F255" s="17"/>
-      <c r="G255" s="17"/>
-      <c r="H255" s="17"/>
-      <c r="I255" s="17"/>
-      <c r="J255" s="17"/>
-      <c r="K255" s="18"/>
+      <c r="B255" s="14"/>
+      <c r="C255" s="14"/>
+      <c r="D255" s="14"/>
+      <c r="E255" s="14"/>
+      <c r="F255" s="14"/>
+      <c r="G255" s="14"/>
+      <c r="H255" s="14"/>
+      <c r="I255" s="14"/>
+      <c r="J255" s="14"/>
+      <c r="K255" s="15"/>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A256" s="10" t="s">
@@ -11793,19 +11782,19 @@
       </c>
     </row>
     <row r="272" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A272" s="16" t="s">
+      <c r="A272" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="B272" s="17"/>
-      <c r="C272" s="17"/>
-      <c r="D272" s="17"/>
-      <c r="E272" s="17"/>
-      <c r="F272" s="17"/>
-      <c r="G272" s="17"/>
-      <c r="H272" s="17"/>
-      <c r="I272" s="17"/>
-      <c r="J272" s="17"/>
-      <c r="K272" s="18"/>
+      <c r="B272" s="14"/>
+      <c r="C272" s="14"/>
+      <c r="D272" s="14"/>
+      <c r="E272" s="14"/>
+      <c r="F272" s="14"/>
+      <c r="G272" s="14"/>
+      <c r="H272" s="14"/>
+      <c r="I272" s="14"/>
+      <c r="J272" s="14"/>
+      <c r="K272" s="15"/>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A273" s="10" t="s">
@@ -12343,19 +12332,19 @@
       </c>
     </row>
     <row r="289" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A289" s="16" t="s">
+      <c r="A289" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="B289" s="17"/>
-      <c r="C289" s="17"/>
-      <c r="D289" s="17"/>
-      <c r="E289" s="17"/>
-      <c r="F289" s="17"/>
-      <c r="G289" s="17"/>
-      <c r="H289" s="17"/>
-      <c r="I289" s="17"/>
-      <c r="J289" s="17"/>
-      <c r="K289" s="18"/>
+      <c r="B289" s="14"/>
+      <c r="C289" s="14"/>
+      <c r="D289" s="14"/>
+      <c r="E289" s="14"/>
+      <c r="F289" s="14"/>
+      <c r="G289" s="14"/>
+      <c r="H289" s="14"/>
+      <c r="I289" s="14"/>
+      <c r="J289" s="14"/>
+      <c r="K289" s="15"/>
     </row>
     <row r="290" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A290" s="10" t="s">
@@ -12894,6 +12883,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
     <mergeCell ref="A289:K289"/>
     <mergeCell ref="A136:K136"/>
     <mergeCell ref="A119:K119"/>
@@ -12910,8 +12901,6 @@
     <mergeCell ref="A68:K68"/>
     <mergeCell ref="A255:K255"/>
     <mergeCell ref="A102:K102"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:XFD1048576">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">

</xml_diff>